<commit_message>
carga dsi unida 3.3
</commit_message>
<xml_diff>
--- a/Ciclo 01/Cuadro de notas.xlsx
+++ b/Ciclo 01/Cuadro de notas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luis Vasquez\Desktop\UES-2026\Ciclo 01\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luizi\OneDrive\Escritorio\UES-2026\Ciclo 01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EC57612-1120-4AFE-B068-2E6F3100DD09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D950189-ABEC-44AD-8E92-2C732CD932B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{8B416A22-FD13-409B-B356-C908504C11D1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8B416A22-FD13-409B-B356-C908504C11D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -29,9 +29,6 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -148,7 +145,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -219,6 +216,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -426,7 +431,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -517,6 +522,11 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="10" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -833,15 +843,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A82A0CD-7BCC-4D99-8D34-01F85165CA32}">
   <dimension ref="A1:N28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="26.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="35" t="s">
         <v>12</v>
       </c>
@@ -861,7 +871,7 @@
       <c r="M2" s="42"/>
       <c r="N2" s="43"/>
     </row>
-    <row r="3" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
@@ -901,7 +911,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
         <v>17</v>
       </c>
@@ -934,13 +944,15 @@
       <c r="L4" s="19">
         <v>0.15</v>
       </c>
-      <c r="M4" s="10"/>
+      <c r="M4" s="10">
+        <v>0</v>
+      </c>
       <c r="N4" s="2">
         <f>+L4*M4</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="27" t="s">
         <v>10</v>
       </c>
@@ -953,14 +965,14 @@
         <v>0</v>
       </c>
       <c r="E5" s="8"/>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="21">
+      <c r="G5" s="28">
         <v>0.1</v>
       </c>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3">
+      <c r="H5" s="2"/>
+      <c r="I5" s="2">
         <f t="shared" ref="I5:I11" si="1">+G5*H5</f>
         <v>0</v>
       </c>
@@ -979,27 +991,27 @@
         <v>0.89999999999999991</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
+    <row r="6" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="23">
+      <c r="B6" s="45">
         <v>0.1</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3">
+      <c r="C6" s="46"/>
+      <c r="D6" s="46">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="E6" s="8"/>
-      <c r="F6" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="G6" s="23">
+      <c r="F6" s="44" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="45">
         <v>0.15</v>
       </c>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3">
+      <c r="H6" s="46"/>
+      <c r="I6" s="46">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1010,13 +1022,15 @@
       <c r="L6" s="23">
         <v>0.05</v>
       </c>
-      <c r="M6" s="13"/>
+      <c r="M6" s="13">
+        <v>0</v>
+      </c>
       <c r="N6" s="3">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="20" t="s">
         <v>11</v>
       </c>
@@ -1047,13 +1061,15 @@
       <c r="L7" s="21">
         <v>0.2</v>
       </c>
-      <c r="M7" s="13"/>
+      <c r="M7" s="13">
+        <v>0</v>
+      </c>
       <c r="N7" s="3">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
         <v>19</v>
       </c>
@@ -1084,13 +1100,15 @@
       <c r="L8" s="23">
         <v>0.1</v>
       </c>
-      <c r="M8" s="13"/>
+      <c r="M8" s="13">
+        <v>0</v>
+      </c>
       <c r="N8" s="3">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="20" t="s">
         <v>20</v>
       </c>
@@ -1121,13 +1139,15 @@
       <c r="L9" s="21">
         <v>0.15</v>
       </c>
-      <c r="M9" s="3"/>
+      <c r="M9" s="3">
+        <v>0</v>
+      </c>
       <c r="N9" s="3">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
         <v>0</v>
       </c>
@@ -1158,13 +1178,15 @@
       <c r="L10" s="23">
         <v>0.2</v>
       </c>
-      <c r="M10" s="3"/>
+      <c r="M10" s="3">
+        <v>0</v>
+      </c>
       <c r="N10" s="3">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" ht="18" x14ac:dyDescent="0.35">
       <c r="A11" s="8"/>
       <c r="B11" s="15"/>
       <c r="C11" s="9"/>
@@ -1193,7 +1215,7 @@
         <v>0.89999999999999991</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -1212,7 +1234,7 @@
       <c r="M12" s="8"/>
       <c r="N12" s="8"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="8"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -1228,7 +1250,7 @@
       <c r="M13" s="8"/>
       <c r="N13" s="8"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="8"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -1244,7 +1266,7 @@
       <c r="M14" s="8"/>
       <c r="N14" s="8"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="8"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -1260,7 +1282,7 @@
       <c r="M15" s="8"/>
       <c r="N15" s="8"/>
     </row>
-    <row r="16" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="8"/>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -1276,7 +1298,7 @@
       <c r="M16" s="8"/>
       <c r="N16" s="8"/>
     </row>
-    <row r="17" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="29" t="s">
         <v>15</v>
       </c>
@@ -1296,7 +1318,7 @@
       <c r="M17" s="8"/>
       <c r="N17" s="8"/>
     </row>
-    <row r="18" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>5</v>
       </c>
@@ -1328,7 +1350,7 @@
       <c r="M18" s="11"/>
       <c r="N18" s="11"/>
     </row>
-    <row r="19" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="18" t="s">
         <v>21</v>
       </c>
@@ -1360,7 +1382,7 @@
       <c r="M19" s="8"/>
       <c r="N19" s="8"/>
     </row>
-    <row r="20" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="27" t="s">
         <v>0</v>
       </c>
@@ -1375,14 +1397,14 @@
         <v>1</v>
       </c>
       <c r="E20" s="8"/>
-      <c r="F20" s="22" t="s">
+      <c r="F20" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G20" s="23">
+      <c r="G20" s="45">
         <v>0.15</v>
       </c>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3">
+      <c r="H20" s="46"/>
+      <c r="I20" s="46">
         <f t="shared" ref="I20:I26" si="4">+G20*H20</f>
         <v>0</v>
       </c>
@@ -1392,7 +1414,7 @@
       <c r="M20" s="8"/>
       <c r="N20" s="8"/>
     </row>
-    <row r="21" spans="1:14" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
         <v>7</v>
       </c>
@@ -1422,7 +1444,7 @@
       <c r="M21" s="8"/>
       <c r="N21" s="8"/>
     </row>
-    <row r="22" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="20" t="s">
         <v>8</v>
       </c>
@@ -1452,7 +1474,7 @@
       <c r="M22" s="8"/>
       <c r="N22" s="8"/>
     </row>
-    <row r="23" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
         <v>22</v>
       </c>
@@ -1482,7 +1504,7 @@
       <c r="M23" s="8"/>
       <c r="N23" s="8"/>
     </row>
-    <row r="24" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="20" t="s">
         <v>25</v>
       </c>
@@ -1512,7 +1534,7 @@
       <c r="M24" s="8"/>
       <c r="N24" s="8"/>
     </row>
-    <row r="25" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="22" t="s">
         <v>26</v>
       </c>
@@ -1542,7 +1564,7 @@
       <c r="M25" s="8"/>
       <c r="N25" s="8"/>
     </row>
-    <row r="26" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" s="20" t="s">
         <v>27</v>
       </c>
@@ -1572,7 +1594,7 @@
       <c r="M26" s="8"/>
       <c r="N26" s="8"/>
     </row>
-    <row r="27" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="22" t="s">
         <v>28</v>
       </c>
@@ -1595,7 +1617,7 @@
       <c r="M27" s="8"/>
       <c r="N27" s="8"/>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="D28" s="17">
         <f>SUM(D19:D27)</f>
         <v>1.5</v>

</xml_diff>